<commit_message>
small fix in sequence diagram
</commit_message>
<xml_diff>
--- a/about/MCS_Fall_Detection.xlsx
+++ b/about/MCS_Fall_Detection.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hayat\Documents\6G\FallDetection_new\_concept_6G_integration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hayat\Documents\6G\FallDetection_new\about\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE78E0D6-C7BE-4D51-A057-03681A93EA81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FC28B2-16AF-4124-9FEF-E07CB517E091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="1" activeTab="1" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
   </bookViews>
@@ -11756,20 +11756,12 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="1000">
+            <a:rPr lang="en-GB" sz="1000" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Fall</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1000" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t> Dashboard</a:t>
+            <a:t>Dashboard</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1000">
             <a:solidFill>
@@ -13445,7 +13437,7 @@
       <xdr:rowOff>167641</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>554935</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>167641</xdr:rowOff>
@@ -13464,7 +13456,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9272346" y="6644641"/>
-          <a:ext cx="5379589" cy="0"/>
+          <a:ext cx="1702111" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>

</xml_diff>